<commit_message>
Add Exam 2 killer
</commit_message>
<xml_diff>
--- a/public/exam project2/TreyResearch.xlsx
+++ b/public/exam project2/TreyResearch.xlsx
@@ -5,13 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\T Irvin Pineda\Desktop\CERTI MO-211\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\T Irvin Pineda\Desktop\mo211-simulator (2)\mo211-simulator\public\exam project2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B25C619E-D2E6-41C3-A99F-28562BA1AAF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <workbookProtection workbookPassword="CF44" lockStructure="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1862112-D641-4589-9A0E-303DACFA7C97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="390" windowWidth="20490" windowHeight="7785" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Fish Survey" sheetId="1" r:id="rId1"/>

</xml_diff>